<commit_message>
Clean HTML report section numbering
</commit_message>
<xml_diff>
--- a/projects/2026-05-fujie-gcard-v1/versions/fujie_gcard_v7_20260630/reports/model_report.xlsx
+++ b/projects/2026-05-fujie-gcard-v1/versions/fujie_gcard_v7_20260630/reports/model_report.xlsx
@@ -1145,7 +1145,7 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>更新日期：2026-06-30；指标来源：当前 run 已注册 train/evaluation artifacts。</t>
+          <t>更新日期：2026-07-01；指标来源：当前 run 已注册 train/evaluation artifacts。</t>
         </is>
       </c>
     </row>
@@ -6490,7 +6490,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
     </row>

</xml_diff>